<commit_message>
Prioritize local Excel matches to find the right part
Search price lists first for the scanned code inside product text,
rank [ВАШ ПРАЙС] above FAPI cross-refs, and document how to raise
hit rate by embedding the barcode in Excel names.

Co-authored-by: omriasolin123456-netizen <omriasolin123456-netizen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/price/format2_name_madel_brand.xlsx
+++ b/price/format2_name_madel_brand.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,6 +541,38 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>4515</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>IGNORE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Шаровая опора 19 мм B3W /361337 PSTB3</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GOLF</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>WXQP</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>&gt;10</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>5000</t>
         </is>
       </c>
     </row>

</xml_diff>